<commit_message>
Timesheet approval Global search and toggle search working.
</commit_message>
<xml_diff>
--- a/EmployeeBillableData_26.xlsx
+++ b/EmployeeBillableData_26.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="178">
   <si>
     <t>EmployeementId</t>
   </si>
@@ -356,15 +356,6 @@
     <t>mitravanu.ray.ap2luat@ap2l.ai</t>
   </si>
   <si>
-    <t>A-240015</t>
-  </si>
-  <si>
-    <t>Prachi Verma</t>
-  </si>
-  <si>
-    <t>prachi.verma.ap2luat@ap2l.ai</t>
-  </si>
-  <si>
     <t>A-240016</t>
   </si>
   <si>
@@ -372,15 +363,6 @@
   </si>
   <si>
     <t>soumyaa.das.ap2luat@ap2l.ai</t>
-  </si>
-  <si>
-    <t>A-240018</t>
-  </si>
-  <si>
-    <t>Subhra Bhanja</t>
-  </si>
-  <si>
-    <t>subhra.bhanja.ap2luat@ap2l.ai</t>
   </si>
   <si>
     <t>A-240043</t>
@@ -642,7 +624,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K52"/>
+  <dimension ref="A1:K50"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="18.55859375" customWidth="true" bestFit="true"/>
@@ -1637,7 +1619,7 @@
         <v>15</v>
       </c>
       <c r="G32" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="H32" t="s">
         <v>17</v>
@@ -1667,13 +1649,13 @@
         <v>15</v>
       </c>
       <c r="G33" t="s">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="H33" t="s">
         <v>17</v>
       </c>
       <c r="I33" t="s">
-        <v>18</v>
+        <v>123</v>
       </c>
       <c r="J33" t="s">
         <v>19</v>
@@ -1681,13 +1663,13 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B34" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C34" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D34"/>
       <c r="E34" t="s">
@@ -1697,7 +1679,7 @@
         <v>15</v>
       </c>
       <c r="G34" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="H34" t="s">
         <v>17</v>
@@ -1711,13 +1693,13 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B35" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C35" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D35"/>
       <c r="E35" t="s">
@@ -1733,7 +1715,7 @@
         <v>17</v>
       </c>
       <c r="I35" t="s">
-        <v>129</v>
+        <v>18</v>
       </c>
       <c r="J35" t="s">
         <v>19</v>
@@ -1757,7 +1739,7 @@
         <v>15</v>
       </c>
       <c r="G36" t="s">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="H36" t="s">
         <v>17</v>
@@ -1823,21 +1805,21 @@
         <v>17</v>
       </c>
       <c r="I38" t="s">
-        <v>18</v>
+        <v>139</v>
       </c>
       <c r="J38" t="s">
-        <v>19</v>
+        <v>44</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B39" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C39" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D39"/>
       <c r="E39" t="s">
@@ -1861,17 +1843,19 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B40" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C40" t="s">
-        <v>144</v>
-      </c>
-      <c r="D40"/>
+        <v>145</v>
+      </c>
+      <c r="D40" t="s">
+        <v>37</v>
+      </c>
       <c r="E40" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="F40" t="s">
         <v>15</v>
@@ -1883,7 +1867,7 @@
         <v>17</v>
       </c>
       <c r="I40" t="s">
-        <v>145</v>
+        <v>69</v>
       </c>
       <c r="J40" t="s">
         <v>44</v>
@@ -1899,9 +1883,11 @@
       <c r="C41" t="s">
         <v>148</v>
       </c>
-      <c r="D41"/>
+      <c r="D41" t="s">
+        <v>13</v>
+      </c>
       <c r="E41" t="s">
-        <v>29</v>
+        <v>96</v>
       </c>
       <c r="F41" t="s">
         <v>15</v>
@@ -1913,7 +1899,7 @@
         <v>17</v>
       </c>
       <c r="I41" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="J41" t="s">
         <v>19</v>
@@ -1921,19 +1907,19 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B42" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C42" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D42" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="E42" t="s">
-        <v>38</v>
+        <v>96</v>
       </c>
       <c r="F42" t="s">
         <v>15</v>
@@ -1945,27 +1931,25 @@
         <v>17</v>
       </c>
       <c r="I42" t="s">
-        <v>69</v>
+        <v>149</v>
       </c>
       <c r="J42" t="s">
-        <v>44</v>
+        <v>19</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B43" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C43" t="s">
-        <v>154</v>
-      </c>
-      <c r="D43" t="s">
-        <v>13</v>
-      </c>
+        <v>155</v>
+      </c>
+      <c r="D43"/>
       <c r="E43" t="s">
-        <v>96</v>
+        <v>29</v>
       </c>
       <c r="F43" t="s">
         <v>15</v>
@@ -1977,7 +1961,7 @@
         <v>17</v>
       </c>
       <c r="I43" t="s">
-        <v>155</v>
+        <v>18</v>
       </c>
       <c r="J43" t="s">
         <v>19</v>
@@ -2003,13 +1987,13 @@
         <v>15</v>
       </c>
       <c r="G44" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="H44" t="s">
         <v>17</v>
       </c>
       <c r="I44" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="J44" t="s">
         <v>19</v>
@@ -2017,17 +2001,19 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B45" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C45" t="s">
-        <v>161</v>
-      </c>
-      <c r="D45"/>
+        <v>162</v>
+      </c>
+      <c r="D45" t="s">
+        <v>13</v>
+      </c>
       <c r="E45" t="s">
-        <v>29</v>
+        <v>96</v>
       </c>
       <c r="F45" t="s">
         <v>15</v>
@@ -2039,7 +2025,7 @@
         <v>17</v>
       </c>
       <c r="I45" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="J45" t="s">
         <v>19</v>
@@ -2047,31 +2033,29 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B46" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C46" t="s">
-        <v>164</v>
-      </c>
-      <c r="D46" t="s">
-        <v>13</v>
-      </c>
+        <v>165</v>
+      </c>
+      <c r="D46"/>
       <c r="E46" t="s">
-        <v>96</v>
+        <v>29</v>
       </c>
       <c r="F46" t="s">
         <v>15</v>
       </c>
       <c r="G46" t="s">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="H46" t="s">
         <v>17</v>
       </c>
       <c r="I46" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="J46" t="s">
         <v>19</v>
@@ -2082,28 +2066,26 @@
         <v>166</v>
       </c>
       <c r="B47" t="s">
+        <v>17</v>
+      </c>
+      <c r="C47" t="s">
         <v>167</v>
       </c>
-      <c r="C47" t="s">
+      <c r="D47"/>
+      <c r="E47" t="s">
+        <v>29</v>
+      </c>
+      <c r="F47" t="s">
+        <v>15</v>
+      </c>
+      <c r="G47" t="s">
         <v>168</v>
       </c>
-      <c r="D47" t="s">
-        <v>13</v>
-      </c>
-      <c r="E47" t="s">
-        <v>96</v>
-      </c>
-      <c r="F47" t="s">
-        <v>15</v>
-      </c>
-      <c r="G47" t="s">
-        <v>33</v>
-      </c>
       <c r="H47" t="s">
         <v>17</v>
       </c>
       <c r="I47" t="s">
-        <v>155</v>
+        <v>18</v>
       </c>
       <c r="J47" t="s">
         <v>19</v>
@@ -2127,13 +2109,13 @@
         <v>15</v>
       </c>
       <c r="G48" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="H48" t="s">
         <v>17</v>
       </c>
       <c r="I48" t="s">
-        <v>165</v>
+        <v>18</v>
       </c>
       <c r="J48" t="s">
         <v>19</v>
@@ -2144,10 +2126,10 @@
         <v>172</v>
       </c>
       <c r="B49" t="s">
-        <v>17</v>
+        <v>173</v>
       </c>
       <c r="C49" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D49"/>
       <c r="E49" t="s">
@@ -2157,7 +2139,7 @@
         <v>15</v>
       </c>
       <c r="G49" t="s">
-        <v>174</v>
+        <v>17</v>
       </c>
       <c r="H49" t="s">
         <v>17</v>
@@ -2179,7 +2161,9 @@
       <c r="C50" t="s">
         <v>177</v>
       </c>
-      <c r="D50"/>
+      <c r="D50" t="s">
+        <v>13</v>
+      </c>
       <c r="E50" t="s">
         <v>29</v>
       </c>
@@ -2187,75 +2171,13 @@
         <v>15</v>
       </c>
       <c r="G50" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="H50" t="s">
         <v>17</v>
       </c>
-      <c r="I50" t="s">
-        <v>18</v>
-      </c>
-      <c r="J50" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="s">
-        <v>178</v>
-      </c>
-      <c r="B51" t="s">
-        <v>179</v>
-      </c>
-      <c r="C51" t="s">
-        <v>180</v>
-      </c>
-      <c r="D51"/>
-      <c r="E51" t="s">
-        <v>29</v>
-      </c>
-      <c r="F51" t="s">
-        <v>15</v>
-      </c>
-      <c r="G51" t="s">
-        <v>17</v>
-      </c>
-      <c r="H51" t="s">
-        <v>17</v>
-      </c>
-      <c r="I51" t="s">
-        <v>18</v>
-      </c>
-      <c r="J51" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="s">
-        <v>181</v>
-      </c>
-      <c r="B52" t="s">
-        <v>182</v>
-      </c>
-      <c r="C52" t="s">
-        <v>183</v>
-      </c>
-      <c r="D52" t="s">
-        <v>13</v>
-      </c>
-      <c r="E52" t="s">
-        <v>29</v>
-      </c>
-      <c r="F52" t="s">
-        <v>15</v>
-      </c>
-      <c r="G52" t="s">
-        <v>33</v>
-      </c>
-      <c r="H52" t="s">
-        <v>17</v>
-      </c>
-      <c r="I52"/>
-      <c r="J52"/>
+      <c r="I50"/>
+      <c r="J50"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
FE Single approve and reject
</commit_message>
<xml_diff>
--- a/EmployeeBillableData_26.xlsx
+++ b/EmployeeBillableData_26.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="176">
   <si>
     <t>EmployeementId</t>
   </si>
@@ -249,12 +249,6 @@
   </si>
   <si>
     <t>aditya.bhowmik.ap2luat@ap2l.ai</t>
-  </si>
-  <si>
-    <t>ATDevOps-TnM-MMFSL-Quiklyz,Products and RND Internal</t>
-  </si>
-  <si>
-    <t>ApMoSys,Mahindra and Mahindra Finance Services Ltd</t>
   </si>
   <si>
     <t>A-240135</t>
@@ -1227,21 +1221,21 @@
         <v>17</v>
       </c>
       <c r="I19" t="s">
-        <v>79</v>
+        <v>18</v>
       </c>
       <c r="J19" t="s">
-        <v>80</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
+        <v>79</v>
+      </c>
+      <c r="B20" t="s">
+        <v>80</v>
+      </c>
+      <c r="C20" t="s">
         <v>81</v>
-      </c>
-      <c r="B20" t="s">
-        <v>82</v>
-      </c>
-      <c r="C20" t="s">
-        <v>83</v>
       </c>
       <c r="D20"/>
       <c r="E20" t="s">
@@ -1265,13 +1259,13 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
+        <v>82</v>
+      </c>
+      <c r="B21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C21" t="s">
         <v>84</v>
-      </c>
-      <c r="B21" t="s">
-        <v>85</v>
-      </c>
-      <c r="C21" t="s">
-        <v>86</v>
       </c>
       <c r="D21"/>
       <c r="E21" t="s">
@@ -1295,13 +1289,13 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
+        <v>85</v>
+      </c>
+      <c r="B22" t="s">
+        <v>86</v>
+      </c>
+      <c r="C22" t="s">
         <v>87</v>
-      </c>
-      <c r="B22" t="s">
-        <v>88</v>
-      </c>
-      <c r="C22" t="s">
-        <v>89</v>
       </c>
       <c r="D22"/>
       <c r="E22" t="s">
@@ -1325,13 +1319,13 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
+        <v>88</v>
+      </c>
+      <c r="B23" t="s">
+        <v>89</v>
+      </c>
+      <c r="C23" t="s">
         <v>90</v>
-      </c>
-      <c r="B23" t="s">
-        <v>91</v>
-      </c>
-      <c r="C23" t="s">
-        <v>92</v>
       </c>
       <c r="D23" t="s">
         <v>13</v>
@@ -1357,19 +1351,19 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
+        <v>91</v>
+      </c>
+      <c r="B24" t="s">
+        <v>92</v>
+      </c>
+      <c r="C24" t="s">
         <v>93</v>
-      </c>
-      <c r="B24" t="s">
-        <v>94</v>
-      </c>
-      <c r="C24" t="s">
-        <v>95</v>
       </c>
       <c r="D24" t="s">
         <v>13</v>
       </c>
       <c r="E24" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F24" t="s">
         <v>15</v>
@@ -1389,13 +1383,13 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
+        <v>95</v>
+      </c>
+      <c r="B25" t="s">
+        <v>96</v>
+      </c>
+      <c r="C25" t="s">
         <v>97</v>
-      </c>
-      <c r="B25" t="s">
-        <v>98</v>
-      </c>
-      <c r="C25" t="s">
-        <v>99</v>
       </c>
       <c r="D25"/>
       <c r="E25" t="s">
@@ -1419,13 +1413,13 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B26" t="s">
         <v>42</v>
       </c>
       <c r="C26" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D26"/>
       <c r="E26" t="s">
@@ -1449,13 +1443,13 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B27" t="s">
         <v>33</v>
       </c>
       <c r="C27" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D27" t="s">
         <v>13</v>
@@ -1473,21 +1467,21 @@
         <v>17</v>
       </c>
       <c r="I27" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="J27" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B28" t="s">
         <v>16</v>
       </c>
       <c r="C28" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D28" t="s">
         <v>13</v>
@@ -1513,13 +1507,13 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
+        <v>106</v>
+      </c>
+      <c r="B29" t="s">
+        <v>107</v>
+      </c>
+      <c r="C29" t="s">
         <v>108</v>
-      </c>
-      <c r="B29" t="s">
-        <v>109</v>
-      </c>
-      <c r="C29" t="s">
-        <v>110</v>
       </c>
       <c r="D29"/>
       <c r="E29" t="s">
@@ -1543,13 +1537,13 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
+        <v>109</v>
+      </c>
+      <c r="B30" t="s">
+        <v>110</v>
+      </c>
+      <c r="C30" t="s">
         <v>111</v>
-      </c>
-      <c r="B30" t="s">
-        <v>112</v>
-      </c>
-      <c r="C30" t="s">
-        <v>113</v>
       </c>
       <c r="D30"/>
       <c r="E30" t="s">
@@ -1573,13 +1567,13 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
+        <v>112</v>
+      </c>
+      <c r="B31" t="s">
+        <v>113</v>
+      </c>
+      <c r="C31" t="s">
         <v>114</v>
-      </c>
-      <c r="B31" t="s">
-        <v>115</v>
-      </c>
-      <c r="C31" t="s">
-        <v>116</v>
       </c>
       <c r="D31"/>
       <c r="E31" t="s">
@@ -1603,13 +1597,13 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
+        <v>115</v>
+      </c>
+      <c r="B32" t="s">
+        <v>116</v>
+      </c>
+      <c r="C32" t="s">
         <v>117</v>
-      </c>
-      <c r="B32" t="s">
-        <v>118</v>
-      </c>
-      <c r="C32" t="s">
-        <v>119</v>
       </c>
       <c r="D32"/>
       <c r="E32" t="s">
@@ -1633,13 +1627,13 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
+        <v>118</v>
+      </c>
+      <c r="B33" t="s">
+        <v>119</v>
+      </c>
+      <c r="C33" t="s">
         <v>120</v>
-      </c>
-      <c r="B33" t="s">
-        <v>121</v>
-      </c>
-      <c r="C33" t="s">
-        <v>122</v>
       </c>
       <c r="D33"/>
       <c r="E33" t="s">
@@ -1655,7 +1649,7 @@
         <v>17</v>
       </c>
       <c r="I33" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="J33" t="s">
         <v>19</v>
@@ -1663,13 +1657,13 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
+        <v>122</v>
+      </c>
+      <c r="B34" t="s">
+        <v>123</v>
+      </c>
+      <c r="C34" t="s">
         <v>124</v>
-      </c>
-      <c r="B34" t="s">
-        <v>125</v>
-      </c>
-      <c r="C34" t="s">
-        <v>126</v>
       </c>
       <c r="D34"/>
       <c r="E34" t="s">
@@ -1693,13 +1687,13 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
+        <v>125</v>
+      </c>
+      <c r="B35" t="s">
+        <v>126</v>
+      </c>
+      <c r="C35" t="s">
         <v>127</v>
-      </c>
-      <c r="B35" t="s">
-        <v>128</v>
-      </c>
-      <c r="C35" t="s">
-        <v>129</v>
       </c>
       <c r="D35"/>
       <c r="E35" t="s">
@@ -1723,13 +1717,13 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
+        <v>128</v>
+      </c>
+      <c r="B36" t="s">
+        <v>129</v>
+      </c>
+      <c r="C36" t="s">
         <v>130</v>
-      </c>
-      <c r="B36" t="s">
-        <v>131</v>
-      </c>
-      <c r="C36" t="s">
-        <v>132</v>
       </c>
       <c r="D36"/>
       <c r="E36" t="s">
@@ -1753,13 +1747,13 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
+        <v>131</v>
+      </c>
+      <c r="B37" t="s">
+        <v>132</v>
+      </c>
+      <c r="C37" t="s">
         <v>133</v>
-      </c>
-      <c r="B37" t="s">
-        <v>134</v>
-      </c>
-      <c r="C37" t="s">
-        <v>135</v>
       </c>
       <c r="D37"/>
       <c r="E37" t="s">
@@ -1783,13 +1777,13 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
+        <v>134</v>
+      </c>
+      <c r="B38" t="s">
+        <v>135</v>
+      </c>
+      <c r="C38" t="s">
         <v>136</v>
-      </c>
-      <c r="B38" t="s">
-        <v>137</v>
-      </c>
-      <c r="C38" t="s">
-        <v>138</v>
       </c>
       <c r="D38"/>
       <c r="E38" t="s">
@@ -1805,7 +1799,7 @@
         <v>17</v>
       </c>
       <c r="I38" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="J38" t="s">
         <v>44</v>
@@ -1813,13 +1807,13 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
+        <v>138</v>
+      </c>
+      <c r="B39" t="s">
+        <v>139</v>
+      </c>
+      <c r="C39" t="s">
         <v>140</v>
-      </c>
-      <c r="B39" t="s">
-        <v>141</v>
-      </c>
-      <c r="C39" t="s">
-        <v>142</v>
       </c>
       <c r="D39"/>
       <c r="E39" t="s">
@@ -1843,13 +1837,13 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
+        <v>141</v>
+      </c>
+      <c r="B40" t="s">
+        <v>142</v>
+      </c>
+      <c r="C40" t="s">
         <v>143</v>
-      </c>
-      <c r="B40" t="s">
-        <v>144</v>
-      </c>
-      <c r="C40" t="s">
-        <v>145</v>
       </c>
       <c r="D40" t="s">
         <v>37</v>
@@ -1875,19 +1869,19 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
+        <v>144</v>
+      </c>
+      <c r="B41" t="s">
+        <v>145</v>
+      </c>
+      <c r="C41" t="s">
         <v>146</v>
-      </c>
-      <c r="B41" t="s">
-        <v>147</v>
-      </c>
-      <c r="C41" t="s">
-        <v>148</v>
       </c>
       <c r="D41" t="s">
         <v>13</v>
       </c>
       <c r="E41" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F41" t="s">
         <v>15</v>
@@ -1899,7 +1893,7 @@
         <v>17</v>
       </c>
       <c r="I41" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="J41" t="s">
         <v>19</v>
@@ -1907,19 +1901,19 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
+        <v>148</v>
+      </c>
+      <c r="B42" t="s">
+        <v>149</v>
+      </c>
+      <c r="C42" t="s">
         <v>150</v>
-      </c>
-      <c r="B42" t="s">
-        <v>151</v>
-      </c>
-      <c r="C42" t="s">
-        <v>152</v>
       </c>
       <c r="D42" t="s">
         <v>13</v>
       </c>
       <c r="E42" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F42" t="s">
         <v>15</v>
@@ -1931,7 +1925,7 @@
         <v>17</v>
       </c>
       <c r="I42" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="J42" t="s">
         <v>19</v>
@@ -1939,13 +1933,13 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
+        <v>151</v>
+      </c>
+      <c r="B43" t="s">
+        <v>152</v>
+      </c>
+      <c r="C43" t="s">
         <v>153</v>
-      </c>
-      <c r="B43" t="s">
-        <v>154</v>
-      </c>
-      <c r="C43" t="s">
-        <v>155</v>
       </c>
       <c r="D43"/>
       <c r="E43" t="s">
@@ -1969,19 +1963,19 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
+        <v>154</v>
+      </c>
+      <c r="B44" t="s">
+        <v>155</v>
+      </c>
+      <c r="C44" t="s">
         <v>156</v>
-      </c>
-      <c r="B44" t="s">
-        <v>157</v>
-      </c>
-      <c r="C44" t="s">
-        <v>158</v>
       </c>
       <c r="D44" t="s">
         <v>13</v>
       </c>
       <c r="E44" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F44" t="s">
         <v>15</v>
@@ -1993,7 +1987,7 @@
         <v>17</v>
       </c>
       <c r="I44" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J44" t="s">
         <v>19</v>
@@ -2001,19 +1995,19 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
+        <v>158</v>
+      </c>
+      <c r="B45" t="s">
+        <v>159</v>
+      </c>
+      <c r="C45" t="s">
         <v>160</v>
-      </c>
-      <c r="B45" t="s">
-        <v>161</v>
-      </c>
-      <c r="C45" t="s">
-        <v>162</v>
       </c>
       <c r="D45" t="s">
         <v>13</v>
       </c>
       <c r="E45" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F45" t="s">
         <v>15</v>
@@ -2025,7 +2019,7 @@
         <v>17</v>
       </c>
       <c r="I45" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="J45" t="s">
         <v>19</v>
@@ -2033,13 +2027,13 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
+        <v>161</v>
+      </c>
+      <c r="B46" t="s">
+        <v>162</v>
+      </c>
+      <c r="C46" t="s">
         <v>163</v>
-      </c>
-      <c r="B46" t="s">
-        <v>164</v>
-      </c>
-      <c r="C46" t="s">
-        <v>165</v>
       </c>
       <c r="D46"/>
       <c r="E46" t="s">
@@ -2055,7 +2049,7 @@
         <v>17</v>
       </c>
       <c r="I46" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J46" t="s">
         <v>19</v>
@@ -2063,13 +2057,13 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B47" t="s">
         <v>17</v>
       </c>
       <c r="C47" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D47"/>
       <c r="E47" t="s">
@@ -2079,7 +2073,7 @@
         <v>15</v>
       </c>
       <c r="G47" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="H47" t="s">
         <v>17</v>
@@ -2093,13 +2087,13 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
+        <v>167</v>
+      </c>
+      <c r="B48" t="s">
+        <v>168</v>
+      </c>
+      <c r="C48" t="s">
         <v>169</v>
-      </c>
-      <c r="B48" t="s">
-        <v>170</v>
-      </c>
-      <c r="C48" t="s">
-        <v>171</v>
       </c>
       <c r="D48"/>
       <c r="E48" t="s">
@@ -2123,13 +2117,13 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
+        <v>170</v>
+      </c>
+      <c r="B49" t="s">
+        <v>171</v>
+      </c>
+      <c r="C49" t="s">
         <v>172</v>
-      </c>
-      <c r="B49" t="s">
-        <v>173</v>
-      </c>
-      <c r="C49" t="s">
-        <v>174</v>
       </c>
       <c r="D49"/>
       <c r="E49" t="s">
@@ -2153,13 +2147,13 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
+        <v>173</v>
+      </c>
+      <c r="B50" t="s">
+        <v>174</v>
+      </c>
+      <c r="C50" t="s">
         <v>175</v>
-      </c>
-      <c r="B50" t="s">
-        <v>176</v>
-      </c>
-      <c r="C50" t="s">
-        <v>177</v>
       </c>
       <c r="D50" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
related changes for previous comming in component ts file
</commit_message>
<xml_diff>
--- a/EmployeeBillableData_26.xlsx
+++ b/EmployeeBillableData_26.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="173">
   <si>
     <t>EmployeementId</t>
   </si>
@@ -116,109 +116,100 @@
     <t>Sonali Thakur</t>
   </si>
   <si>
-    <t>A-23358</t>
-  </si>
-  <si>
-    <t>Abinash Sahoo</t>
-  </si>
-  <si>
-    <t>abinash.sahoo.ap2luat@ap2l.ai</t>
+    <t>A-23393</t>
+  </si>
+  <si>
+    <t>Ajay Jaiswal</t>
+  </si>
+  <si>
+    <t>ajay.jaiswal.ap2luat@ap2l.ai</t>
+  </si>
+  <si>
+    <t>Pritiranjan Das</t>
+  </si>
+  <si>
+    <t>DEV-FA-MON-ertyu-sdbv,Products and RND Internal</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Aniruddha,ApMoSys</t>
+  </si>
+  <si>
+    <t>A-240009</t>
+  </si>
+  <si>
+    <t>Ayush Anurag Mallick</t>
+  </si>
+  <si>
+    <t>ayush.mallick.ap2luat@ap2l.ai</t>
+  </si>
+  <si>
+    <t>A-240010</t>
+  </si>
+  <si>
+    <t>Tulya Keshab Nayak</t>
+  </si>
+  <si>
+    <t>tulya.nayak.ap2luat@ap2l.ai</t>
+  </si>
+  <si>
+    <t>A-240013</t>
+  </si>
+  <si>
+    <t>Rohan Jyoti Mishra</t>
+  </si>
+  <si>
+    <t>rohan.mishra.ap2luat@ap2l.ai</t>
+  </si>
+  <si>
+    <t>A-240056</t>
+  </si>
+  <si>
+    <t>Sachidananda Mallick</t>
+  </si>
+  <si>
+    <t>sachidananda.mallick.ap2luat@ap2l.ai</t>
+  </si>
+  <si>
+    <t>A-240070</t>
+  </si>
+  <si>
+    <t>Jai Tembhare</t>
+  </si>
+  <si>
+    <t>jai.tembhare.ap2luat@ap2l.ai</t>
+  </si>
+  <si>
+    <t>A-240085</t>
+  </si>
+  <si>
+    <t>Aditya Singh</t>
+  </si>
+  <si>
+    <t>aditya.singh.ap2luat@ap2l.ai</t>
+  </si>
+  <si>
+    <t>A-240086</t>
+  </si>
+  <si>
+    <t>Saksham Budhadev</t>
+  </si>
+  <si>
+    <t>saksham.budhadev.ap2luat@ap2l.ai</t>
+  </si>
+  <si>
+    <t>A-240100</t>
+  </si>
+  <si>
+    <t>Adrija Saha</t>
+  </si>
+  <si>
+    <t>adrija.saha.ap2luat@ap2l.ai</t>
   </si>
   <si>
     <t>Yes</t>
   </si>
   <si>
     <t>TNM</t>
-  </si>
-  <si>
-    <t>A-23393</t>
-  </si>
-  <si>
-    <t>Ajay Jaiswal</t>
-  </si>
-  <si>
-    <t>ajay.jaiswal.ap2luat@ap2l.ai</t>
-  </si>
-  <si>
-    <t>Pritiranjan Das</t>
-  </si>
-  <si>
-    <t>DEV-FA-MON-ertyu-sdbv,Products and RND Internal</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Aniruddha,ApMoSys</t>
-  </si>
-  <si>
-    <t>A-240009</t>
-  </si>
-  <si>
-    <t>Ayush Anurag Mallick</t>
-  </si>
-  <si>
-    <t>ayush.mallick.ap2luat@ap2l.ai</t>
-  </si>
-  <si>
-    <t>A-240010</t>
-  </si>
-  <si>
-    <t>Tulya Keshab Nayak</t>
-  </si>
-  <si>
-    <t>tulya.nayak.ap2luat@ap2l.ai</t>
-  </si>
-  <si>
-    <t>A-240013</t>
-  </si>
-  <si>
-    <t>Rohan Jyoti Mishra</t>
-  </si>
-  <si>
-    <t>rohan.mishra.ap2luat@ap2l.ai</t>
-  </si>
-  <si>
-    <t>A-240056</t>
-  </si>
-  <si>
-    <t>Sachidananda Mallick</t>
-  </si>
-  <si>
-    <t>sachidananda.mallick.ap2luat@ap2l.ai</t>
-  </si>
-  <si>
-    <t>A-240070</t>
-  </si>
-  <si>
-    <t>Jai Tembhare</t>
-  </si>
-  <si>
-    <t>jai.tembhare.ap2luat@ap2l.ai</t>
-  </si>
-  <si>
-    <t>A-240085</t>
-  </si>
-  <si>
-    <t>Aditya Singh</t>
-  </si>
-  <si>
-    <t>aditya.singh.ap2luat@ap2l.ai</t>
-  </si>
-  <si>
-    <t>A-240086</t>
-  </si>
-  <si>
-    <t>Saksham Budhadev</t>
-  </si>
-  <si>
-    <t>saksham.budhadev.ap2luat@ap2l.ai</t>
-  </si>
-  <si>
-    <t>A-240100</t>
-  </si>
-  <si>
-    <t>Adrija Saha</t>
-  </si>
-  <si>
-    <t>adrija.saha.ap2luat@ap2l.ai</t>
   </si>
   <si>
     <t>Products and RND Internal,SA - AC - TNM - ertyu - ISHINE-API-TEST</t>
@@ -618,7 +609,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K50"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="18.55859375" customWidth="true" bestFit="true"/>
@@ -834,40 +825,38 @@
         <v>36</v>
       </c>
       <c r="D7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" t="s">
         <v>37</v>
       </c>
-      <c r="E7" t="s">
+      <c r="H7" t="s">
+        <v>17</v>
+      </c>
+      <c r="I7" t="s">
         <v>38</v>
       </c>
-      <c r="F7" t="s">
-        <v>15</v>
-      </c>
-      <c r="G7" t="s">
-        <v>33</v>
-      </c>
-      <c r="H7" t="s">
-        <v>17</v>
-      </c>
-      <c r="I7" t="s">
-        <v>18</v>
-      </c>
       <c r="J7" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>41</v>
-      </c>
-      <c r="D8" t="s">
-        <v>13</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="D8"/>
       <c r="E8" t="s">
         <v>29</v>
       </c>
@@ -875,31 +864,33 @@
         <v>15</v>
       </c>
       <c r="G8" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="H8" t="s">
         <v>17</v>
       </c>
       <c r="I8" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="J8" t="s">
-        <v>44</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" t="s">
         <v>45</v>
       </c>
-      <c r="B9" t="s">
-        <v>46</v>
-      </c>
-      <c r="C9" t="s">
-        <v>47</v>
-      </c>
-      <c r="D9"/>
+      <c r="D9" t="s">
+        <v>13</v>
+      </c>
       <c r="E9" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F9" t="s">
         <v>15</v>
@@ -919,13 +910,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
+        <v>46</v>
+      </c>
+      <c r="B10" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" t="s">
         <v>48</v>
-      </c>
-      <c r="B10" t="s">
-        <v>49</v>
-      </c>
-      <c r="C10" t="s">
-        <v>50</v>
       </c>
       <c r="D10" t="s">
         <v>13</v>
@@ -951,25 +942,23 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B11" t="s">
+        <v>50</v>
+      </c>
+      <c r="C11" t="s">
         <v>51</v>
       </c>
-      <c r="B11" t="s">
-        <v>52</v>
-      </c>
-      <c r="C11" t="s">
-        <v>53</v>
-      </c>
-      <c r="D11" t="s">
-        <v>13</v>
-      </c>
+      <c r="D11"/>
       <c r="E11" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F11" t="s">
         <v>15</v>
       </c>
       <c r="G11" t="s">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="H11" t="s">
         <v>17</v>
@@ -983,13 +972,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
+        <v>52</v>
+      </c>
+      <c r="B12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" t="s">
         <v>54</v>
-      </c>
-      <c r="B12" t="s">
-        <v>55</v>
-      </c>
-      <c r="C12" t="s">
-        <v>56</v>
       </c>
       <c r="D12"/>
       <c r="E12" t="s">
@@ -999,7 +988,7 @@
         <v>15</v>
       </c>
       <c r="G12" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H12" t="s">
         <v>17</v>
@@ -1013,13 +1002,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B13" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13" t="s">
         <v>57</v>
-      </c>
-      <c r="B13" t="s">
-        <v>58</v>
-      </c>
-      <c r="C13" t="s">
-        <v>59</v>
       </c>
       <c r="D13"/>
       <c r="E13" t="s">
@@ -1029,7 +1018,7 @@
         <v>15</v>
       </c>
       <c r="G13" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="H13" t="s">
         <v>17</v>
@@ -1043,13 +1032,13 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
+        <v>58</v>
+      </c>
+      <c r="B14" t="s">
+        <v>59</v>
+      </c>
+      <c r="C14" t="s">
         <v>60</v>
-      </c>
-      <c r="B14" t="s">
-        <v>61</v>
-      </c>
-      <c r="C14" t="s">
-        <v>62</v>
       </c>
       <c r="D14"/>
       <c r="E14" t="s">
@@ -1073,17 +1062,19 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
+        <v>61</v>
+      </c>
+      <c r="B15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C15" t="s">
         <v>63</v>
       </c>
-      <c r="B15" t="s">
+      <c r="D15" t="s">
         <v>64</v>
       </c>
-      <c r="C15" t="s">
+      <c r="E15" t="s">
         <v>65</v>
-      </c>
-      <c r="D15"/>
-      <c r="E15" t="s">
-        <v>29</v>
       </c>
       <c r="F15" t="s">
         <v>15</v>
@@ -1095,27 +1086,27 @@
         <v>17</v>
       </c>
       <c r="I15" t="s">
-        <v>18</v>
+        <v>66</v>
       </c>
       <c r="J15" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B16" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C16" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D16" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="E16" t="s">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="F16" t="s">
         <v>15</v>
@@ -1127,10 +1118,10 @@
         <v>17</v>
       </c>
       <c r="I16" t="s">
-        <v>69</v>
+        <v>18</v>
       </c>
       <c r="J16" t="s">
-        <v>44</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17">
@@ -1143,11 +1134,9 @@
       <c r="C17" t="s">
         <v>72</v>
       </c>
-      <c r="D17" t="s">
-        <v>13</v>
-      </c>
+      <c r="D17"/>
       <c r="E17" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F17" t="s">
         <v>15</v>
@@ -1175,9 +1164,11 @@
       <c r="C18" t="s">
         <v>75</v>
       </c>
-      <c r="D18"/>
+      <c r="D18" t="s">
+        <v>13</v>
+      </c>
       <c r="E18" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F18" t="s">
         <v>15</v>
@@ -1205,17 +1196,15 @@
       <c r="C19" t="s">
         <v>78</v>
       </c>
-      <c r="D19" t="s">
-        <v>13</v>
-      </c>
+      <c r="D19"/>
       <c r="E19" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F19" t="s">
         <v>15</v>
       </c>
       <c r="G19" t="s">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="H19" t="s">
         <v>17</v>
@@ -1245,7 +1234,7 @@
         <v>15</v>
       </c>
       <c r="G20" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="H20" t="s">
         <v>17</v>
@@ -1275,7 +1264,7 @@
         <v>15</v>
       </c>
       <c r="G21" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H21" t="s">
         <v>17</v>
@@ -1297,9 +1286,11 @@
       <c r="C22" t="s">
         <v>87</v>
       </c>
-      <c r="D22"/>
+      <c r="D22" t="s">
+        <v>13</v>
+      </c>
       <c r="E22" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F22" t="s">
         <v>15</v>
@@ -1331,13 +1322,13 @@
         <v>13</v>
       </c>
       <c r="E23" t="s">
-        <v>14</v>
+        <v>91</v>
       </c>
       <c r="F23" t="s">
         <v>15</v>
       </c>
       <c r="G23" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="H23" t="s">
         <v>17</v>
@@ -1351,25 +1342,23 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B24" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C24" t="s">
-        <v>93</v>
-      </c>
-      <c r="D24" t="s">
-        <v>13</v>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="D24"/>
       <c r="E24" t="s">
-        <v>94</v>
+        <v>29</v>
       </c>
       <c r="F24" t="s">
         <v>15</v>
       </c>
       <c r="G24" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="H24" t="s">
         <v>17</v>
@@ -1386,10 +1375,10 @@
         <v>95</v>
       </c>
       <c r="B25" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" t="s">
         <v>96</v>
-      </c>
-      <c r="C25" t="s">
-        <v>97</v>
       </c>
       <c r="D25"/>
       <c r="E25" t="s">
@@ -1399,7 +1388,7 @@
         <v>15</v>
       </c>
       <c r="G25" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H25" t="s">
         <v>17</v>
@@ -1413,43 +1402,45 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
+        <v>97</v>
+      </c>
+      <c r="B26" t="s">
+        <v>33</v>
+      </c>
+      <c r="C26" t="s">
         <v>98</v>
       </c>
-      <c r="B26" t="s">
-        <v>42</v>
-      </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
+        <v>13</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>15</v>
+      </c>
+      <c r="G26" t="s">
+        <v>17</v>
+      </c>
+      <c r="H26" t="s">
+        <v>17</v>
+      </c>
+      <c r="I26" t="s">
         <v>99</v>
       </c>
-      <c r="D26"/>
-      <c r="E26" t="s">
-        <v>29</v>
-      </c>
-      <c r="F26" t="s">
-        <v>15</v>
-      </c>
-      <c r="G26" t="s">
-        <v>17</v>
-      </c>
-      <c r="H26" t="s">
-        <v>17</v>
-      </c>
-      <c r="I26" t="s">
-        <v>18</v>
-      </c>
       <c r="J26" t="s">
-        <v>19</v>
+        <v>100</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B27" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="C27" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D27" t="s">
         <v>13</v>
@@ -1467,33 +1458,31 @@
         <v>17</v>
       </c>
       <c r="I27" t="s">
-        <v>102</v>
+        <v>18</v>
       </c>
       <c r="J27" t="s">
-        <v>103</v>
+        <v>19</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
+        <v>103</v>
+      </c>
+      <c r="B28" t="s">
         <v>104</v>
-      </c>
-      <c r="B28" t="s">
-        <v>16</v>
       </c>
       <c r="C28" t="s">
         <v>105</v>
       </c>
-      <c r="D28" t="s">
-        <v>13</v>
-      </c>
+      <c r="D28"/>
       <c r="E28" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F28" t="s">
         <v>15</v>
       </c>
       <c r="G28" t="s">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="H28" t="s">
         <v>17</v>
@@ -1523,7 +1512,7 @@
         <v>15</v>
       </c>
       <c r="G29" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="H29" t="s">
         <v>17</v>
@@ -1553,7 +1542,7 @@
         <v>15</v>
       </c>
       <c r="G30" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H30" t="s">
         <v>17</v>
@@ -1583,7 +1572,7 @@
         <v>15</v>
       </c>
       <c r="G31" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="H31" t="s">
         <v>17</v>
@@ -1619,7 +1608,7 @@
         <v>17</v>
       </c>
       <c r="I32" t="s">
-        <v>18</v>
+        <v>118</v>
       </c>
       <c r="J32" t="s">
         <v>19</v>
@@ -1627,13 +1616,13 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B33" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C33" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D33"/>
       <c r="E33" t="s">
@@ -1643,13 +1632,13 @@
         <v>15</v>
       </c>
       <c r="G33" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="H33" t="s">
         <v>17</v>
       </c>
       <c r="I33" t="s">
-        <v>121</v>
+        <v>18</v>
       </c>
       <c r="J33" t="s">
         <v>19</v>
@@ -1673,7 +1662,7 @@
         <v>15</v>
       </c>
       <c r="G34" t="s">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="H34" t="s">
         <v>17</v>
@@ -1769,21 +1758,21 @@
         <v>17</v>
       </c>
       <c r="I37" t="s">
-        <v>18</v>
+        <v>134</v>
       </c>
       <c r="J37" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B38" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C38" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D38"/>
       <c r="E38" t="s">
@@ -1799,10 +1788,10 @@
         <v>17</v>
       </c>
       <c r="I38" t="s">
-        <v>137</v>
+        <v>18</v>
       </c>
       <c r="J38" t="s">
-        <v>44</v>
+        <v>19</v>
       </c>
     </row>
     <row r="39">
@@ -1815,9 +1804,11 @@
       <c r="C39" t="s">
         <v>140</v>
       </c>
-      <c r="D39"/>
+      <c r="D39" t="s">
+        <v>64</v>
+      </c>
       <c r="E39" t="s">
-        <v>29</v>
+        <v>65</v>
       </c>
       <c r="F39" t="s">
         <v>15</v>
@@ -1829,10 +1820,10 @@
         <v>17</v>
       </c>
       <c r="I39" t="s">
-        <v>18</v>
+        <v>66</v>
       </c>
       <c r="J39" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
     </row>
     <row r="40">
@@ -1846,10 +1837,10 @@
         <v>143</v>
       </c>
       <c r="D40" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="E40" t="s">
-        <v>38</v>
+        <v>91</v>
       </c>
       <c r="F40" t="s">
         <v>15</v>
@@ -1861,27 +1852,27 @@
         <v>17</v>
       </c>
       <c r="I40" t="s">
-        <v>69</v>
+        <v>144</v>
       </c>
       <c r="J40" t="s">
-        <v>44</v>
+        <v>19</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B41" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C41" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D41" t="s">
         <v>13</v>
       </c>
       <c r="E41" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="F41" t="s">
         <v>15</v>
@@ -1893,7 +1884,7 @@
         <v>17</v>
       </c>
       <c r="I41" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="J41" t="s">
         <v>19</v>
@@ -1909,11 +1900,9 @@
       <c r="C42" t="s">
         <v>150</v>
       </c>
-      <c r="D42" t="s">
-        <v>13</v>
-      </c>
+      <c r="D42"/>
       <c r="E42" t="s">
-        <v>94</v>
+        <v>29</v>
       </c>
       <c r="F42" t="s">
         <v>15</v>
@@ -1925,7 +1914,7 @@
         <v>17</v>
       </c>
       <c r="I42" t="s">
-        <v>147</v>
+        <v>18</v>
       </c>
       <c r="J42" t="s">
         <v>19</v>
@@ -1941,21 +1930,23 @@
       <c r="C43" t="s">
         <v>153</v>
       </c>
-      <c r="D43"/>
+      <c r="D43" t="s">
+        <v>13</v>
+      </c>
       <c r="E43" t="s">
-        <v>29</v>
+        <v>91</v>
       </c>
       <c r="F43" t="s">
         <v>15</v>
       </c>
       <c r="G43" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="H43" t="s">
         <v>17</v>
       </c>
       <c r="I43" t="s">
-        <v>18</v>
+        <v>154</v>
       </c>
       <c r="J43" t="s">
         <v>19</v>
@@ -1963,31 +1954,31 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B44" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C44" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D44" t="s">
         <v>13</v>
       </c>
       <c r="E44" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="F44" t="s">
         <v>15</v>
       </c>
       <c r="G44" t="s">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="H44" t="s">
         <v>17</v>
       </c>
       <c r="I44" t="s">
-        <v>157</v>
+        <v>144</v>
       </c>
       <c r="J44" t="s">
         <v>19</v>
@@ -2003,11 +1994,9 @@
       <c r="C45" t="s">
         <v>160</v>
       </c>
-      <c r="D45" t="s">
-        <v>13</v>
-      </c>
+      <c r="D45"/>
       <c r="E45" t="s">
-        <v>94</v>
+        <v>29</v>
       </c>
       <c r="F45" t="s">
         <v>15</v>
@@ -2019,7 +2008,7 @@
         <v>17</v>
       </c>
       <c r="I45" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="J45" t="s">
         <v>19</v>
@@ -2030,10 +2019,10 @@
         <v>161</v>
       </c>
       <c r="B46" t="s">
+        <v>17</v>
+      </c>
+      <c r="C46" t="s">
         <v>162</v>
-      </c>
-      <c r="C46" t="s">
-        <v>163</v>
       </c>
       <c r="D46"/>
       <c r="E46" t="s">
@@ -2043,13 +2032,13 @@
         <v>15</v>
       </c>
       <c r="G46" t="s">
-        <v>33</v>
+        <v>163</v>
       </c>
       <c r="H46" t="s">
         <v>17</v>
       </c>
       <c r="I46" t="s">
-        <v>157</v>
+        <v>18</v>
       </c>
       <c r="J46" t="s">
         <v>19</v>
@@ -2060,10 +2049,10 @@
         <v>164</v>
       </c>
       <c r="B47" t="s">
-        <v>17</v>
+        <v>165</v>
       </c>
       <c r="C47" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D47"/>
       <c r="E47" t="s">
@@ -2073,7 +2062,7 @@
         <v>15</v>
       </c>
       <c r="G47" t="s">
-        <v>166</v>
+        <v>17</v>
       </c>
       <c r="H47" t="s">
         <v>17</v>
@@ -2125,7 +2114,9 @@
       <c r="C49" t="s">
         <v>172</v>
       </c>
-      <c r="D49"/>
+      <c r="D49" t="s">
+        <v>13</v>
+      </c>
       <c r="E49" t="s">
         <v>29</v>
       </c>
@@ -2133,45 +2124,13 @@
         <v>15</v>
       </c>
       <c r="G49" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="H49" t="s">
         <v>17</v>
       </c>
-      <c r="I49" t="s">
-        <v>18</v>
-      </c>
-      <c r="J49" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="s">
-        <v>173</v>
-      </c>
-      <c r="B50" t="s">
-        <v>174</v>
-      </c>
-      <c r="C50" t="s">
-        <v>175</v>
-      </c>
-      <c r="D50" t="s">
-        <v>13</v>
-      </c>
-      <c r="E50" t="s">
-        <v>29</v>
-      </c>
-      <c r="F50" t="s">
-        <v>15</v>
-      </c>
-      <c r="G50" t="s">
-        <v>33</v>
-      </c>
-      <c r="H50" t="s">
-        <v>17</v>
-      </c>
-      <c r="I50"/>
-      <c r="J50"/>
+      <c r="I49"/>
+      <c r="J49"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
Reimbursement Dashboard Access For all
</commit_message>
<xml_diff>
--- a/EmployeeBillableData_26.xlsx
+++ b/EmployeeBillableData_26.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="718" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="718" uniqueCount="240">
   <si>
     <t>EmployeementId</t>
   </si>
@@ -350,6 +350,9 @@
     <t>tanisha.tanmayee.ap2luat@ap2l.ai</t>
   </si>
   <si>
+    <t>Malaya Ranjan Dalai</t>
+  </si>
+  <si>
     <t>A-260003</t>
   </si>
   <si>
@@ -437,7 +440,7 @@
     <t>abhishek.acharya.ap2luat@ap2l.ai</t>
   </si>
   <si>
-    <t>Shadow</t>
+    <t>Fixed Cost</t>
   </si>
   <si>
     <t>RND - FC -FDC -Apmosys Netraa APM Licenses &amp; Implementation</t>
@@ -1802,7 +1805,7 @@
         <v>15</v>
       </c>
       <c r="G31" t="s">
-        <v>16</v>
+        <v>112</v>
       </c>
       <c r="H31" t="s">
         <v>17</v>
@@ -1816,13 +1819,13 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B32" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C32" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D32" t="s">
         <v>13</v>
@@ -1848,13 +1851,13 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B33" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C33" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D33" t="s">
         <v>13</v>
@@ -1880,13 +1883,13 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B34" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C34" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D34" t="s">
         <v>13</v>
@@ -1912,13 +1915,13 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B35" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C35" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D35" t="s">
         <v>13</v>
@@ -1944,13 +1947,13 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B36" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C36" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D36" t="s">
         <v>13</v>
@@ -1976,13 +1979,13 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B37" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C37" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D37" t="s">
         <v>13</v>
@@ -2008,13 +2011,13 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B38" t="s">
         <v>48</v>
       </c>
       <c r="C38" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D38" t="s">
         <v>13</v>
@@ -2040,13 +2043,13 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B39" t="s">
         <v>61</v>
       </c>
       <c r="C39" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D39" t="s">
         <v>13</v>
@@ -2072,13 +2075,13 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B40" t="s">
         <v>16</v>
       </c>
       <c r="C40" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D40" t="s">
         <v>13</v>
@@ -2104,13 +2107,13 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B41" t="s">
         <v>35</v>
       </c>
       <c r="C41" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D41" t="s">
         <v>13</v>
@@ -2136,19 +2139,19 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B42" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C42" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D42" t="s">
         <v>13</v>
       </c>
       <c r="E42" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F42" t="s">
         <v>15</v>
@@ -2160,21 +2163,21 @@
         <v>17</v>
       </c>
       <c r="I42" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="J42" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B43" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C43" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D43" t="s">
         <v>13</v>
@@ -2200,13 +2203,13 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B44" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C44" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D44" t="s">
         <v>13</v>
@@ -2232,13 +2235,13 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B45" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C45" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D45" t="s">
         <v>13</v>
@@ -2264,13 +2267,13 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B46" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C46" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D46" t="s">
         <v>13</v>
@@ -2296,13 +2299,13 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B47" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C47" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D47" t="s">
         <v>13</v>
@@ -2328,13 +2331,13 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B48" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C48" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D48" t="s">
         <v>13</v>
@@ -2360,13 +2363,13 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B49" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C49" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D49" t="s">
         <v>13</v>
@@ -2392,13 +2395,13 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B50" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C50" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D50" t="s">
         <v>13</v>
@@ -2424,13 +2427,13 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B51" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C51" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D51" t="s">
         <v>13</v>
@@ -2456,13 +2459,13 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B52" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C52" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D52" t="s">
         <v>13</v>
@@ -2488,13 +2491,13 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B53" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C53" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D53" t="s">
         <v>13</v>
@@ -2520,13 +2523,13 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B54" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C54" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D54" t="s">
         <v>13</v>
@@ -2552,13 +2555,13 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B55" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C55" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D55" t="s">
         <v>13</v>
@@ -2584,13 +2587,13 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B56" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C56" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D56" t="s">
         <v>13</v>
@@ -2616,13 +2619,13 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B57" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C57" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D57" t="s">
         <v>13</v>
@@ -2648,13 +2651,13 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B58" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C58" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D58" t="s">
         <v>13</v>
@@ -2680,13 +2683,13 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B59" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C59" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D59" t="s">
         <v>13</v>
@@ -2712,13 +2715,13 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B60" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C60" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D60" t="s">
         <v>13</v>
@@ -2744,19 +2747,19 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B61" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C61" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D61" t="s">
         <v>13</v>
       </c>
       <c r="E61" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F61" t="s">
         <v>15</v>
@@ -2768,7 +2771,7 @@
         <v>17</v>
       </c>
       <c r="I61" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="J61" t="s">
         <v>19</v>
@@ -2776,13 +2779,13 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B62" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C62" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D62" t="s">
         <v>13</v>
@@ -2808,13 +2811,13 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B63" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C63" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D63" t="s">
         <v>13</v>
@@ -2840,13 +2843,13 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B64" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C64" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D64" t="s">
         <v>13</v>
@@ -2872,19 +2875,19 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B65" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C65" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D65" t="s">
         <v>13</v>
       </c>
       <c r="E65" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F65" t="s">
         <v>15</v>
@@ -2896,7 +2899,7 @@
         <v>17</v>
       </c>
       <c r="I65" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="J65" t="s">
         <v>19</v>
@@ -2904,19 +2907,19 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B66" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C66" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D66" t="s">
         <v>13</v>
       </c>
       <c r="E66" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F66" t="s">
         <v>15</v>
@@ -2928,7 +2931,7 @@
         <v>17</v>
       </c>
       <c r="I66" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J66" t="s">
         <v>19</v>
@@ -2936,13 +2939,13 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B67" t="s">
         <v>17</v>
       </c>
       <c r="C67" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D67" t="s">
         <v>13</v>
@@ -2954,7 +2957,7 @@
         <v>15</v>
       </c>
       <c r="G67" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="H67" t="s">
         <v>17</v>
@@ -2964,13 +2967,13 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B68" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C68" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D68" t="s">
         <v>13</v>
@@ -2982,7 +2985,7 @@
         <v>15</v>
       </c>
       <c r="G68" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="H68" t="s">
         <v>17</v>
@@ -2996,13 +2999,13 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B69" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C69" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D69" t="s">
         <v>13</v>
@@ -3028,13 +3031,13 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B70" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C70" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D70" t="s">
         <v>13</v>
@@ -3060,13 +3063,13 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B71" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C71" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D71" t="s">
         <v>13</v>
@@ -3092,13 +3095,13 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B72" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C72" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D72" t="s">
         <v>13</v>

</xml_diff>